<commit_message>
Bổ sung giá liên quan và ước lượng giá cho các thiết bị chưa có giá; thêm phương án cắt giảm
- Đông khô: dùng giá Eyela FDU-2110 (cùng thông số chính FDL-2000); tủ đông: giá tủ -30 °C theo phương án nâng cấp
- 12 hạng mục ước lượng theo mặt bằng giá thị trường VN, ghi khoảng giá và căn cứ
- Tổng 28 hạng mục khoảng 24,8 tỷ; sheet Phương án cắt giảm khoảng 14,45 tỷ
- Sửa nhận xét Corrtest CS310X Option C (đúng là 8 kênh, 1 EIS) trong báo cáo và bản đánh dấu

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLkhnZKuapW5Zj7yjV8vMu
</commit_message>
<xml_diff>
--- a/Du an PTN cao hoc Hoa hoc/Doi sanh gia thiet bi (Net-zero, G9, 4 Thuoc).xlsx
+++ b/Du an PTN cao hoc Hoa hoc/Doi sanh gia thiet bi (Net-zero, G9, 4 Thuoc).xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đối sánh giá" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề xuất bổ sung" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chú giải" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phương án cắt giảm" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề xuất bổ sung" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chú giải" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -59,12 +60,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -99,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,9 +118,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -512,13 +510,13 @@
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
   </cols>
@@ -541,7 +539,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Mức tương đồng về giá</t>
+          <t>Loại giá</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -571,12 +569,12 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Giá tham khảo "Một phần" (chưa cộng)</t>
+          <t>Khoảng ước lượng (đồng)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Căn cứ / ghi chú</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -629,7 +627,7 @@
         <f>IF(H2="","",C2*H2)</f>
         <v/>
       </c>
-      <c r="J2" s="4" t="n"/>
+      <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Tủ hút khí độc BLH18 Phượng Hải (cùng hãng). Nếu lấy đúng loại 1600 mm có màng lọc: tệp G9, sheet "2 CNVS&amp;G", dòng 284 = 220.000.000.</t>
@@ -681,7 +679,7 @@
         <f>IF(H3="","",C3*H3)</f>
         <v/>
       </c>
-      <c r="J3" s="4" t="n"/>
+      <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Cùng model BCE224i-1S Sartorius.</t>
@@ -737,7 +735,7 @@
         <f>IF(H4="","",C4*H4)</f>
         <v/>
       </c>
-      <c r="J4" s="4" t="n"/>
+      <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Cân 2 số lẻ BCE2202i (2.200 g/0,01 g); đề cương là SPX6201 (6.200 g/0,1 g).</t>
@@ -793,7 +791,7 @@
         <f>IF(H5="","",C5*H5)</f>
         <v/>
       </c>
-      <c r="J5" s="4" t="n"/>
+      <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Máy khuấy từ gia nhiệt nhỏ (IKA C-MAG HS 7 theo sheet Append1).</t>
@@ -849,7 +847,7 @@
         <f>IF(H6="","",C6*H6)</f>
         <v/>
       </c>
-      <c r="J6" s="4" t="n"/>
+      <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Bể rửa siêu âm có gia nhiệt (Elma S10H, khoảng 10 L).</t>
@@ -905,7 +903,7 @@
         <f>IF(H7="","",C7*H7)</f>
         <v/>
       </c>
-      <c r="J7" s="4" t="n"/>
+      <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Cùng model Memmert UN55.</t>
@@ -961,7 +959,7 @@
         <f>IF(H8="","",C8*H8)</f>
         <v/>
       </c>
-      <c r="J8" s="4" t="n"/>
+      <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Tủ lạnh gia dụng loại lớn (Panasonic 550 L), lớn hơn 340 L trong đề cương. Nếu đổi sang tủ chống cháy nổ thì giá này không dùng được.</t>
@@ -992,7 +990,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Giá liên quan</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1010,17 +1008,17 @@
           <t>Tủ lạnh âm - 30°C — Tủ lạnh âm - 30°C</t>
         </is>
       </c>
-      <c r="H9" s="7" t="n"/>
+      <c r="H9" s="4" t="n">
+        <v>148800000</v>
+      </c>
       <c r="I9" s="4">
         <f>IF(H9="","",C9*H9)</f>
         <v/>
       </c>
-      <c r="J9" s="4" t="n">
-        <v>148800000</v>
-      </c>
+      <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Tủ âm -30 °C PHC (tủ phòng thí nghiệm), cao cấp hơn tủ đông gia dụng -18 °C; phù hợp với góp ý nâng cấp. Chưa cộng vào tổng.</t>
+          <t>Dùng giá tủ âm -30 °C PHC (tủ phòng thí nghiệm) theo phương án nâng cấp đã góp ý. Nếu giữ tủ đông gia dụng 252 L như đề cương: khoảng 8–12 triệu.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1073,7 +1071,7 @@
         <f>IF(H10="","",C10*H10)</f>
         <v/>
       </c>
-      <c r="J10" s="4" t="n"/>
+      <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Cùng model Hamilton WSC/4D (giá ở sheet tổng hợp Append1, số tròn).</t>
@@ -1102,23 +1100,33 @@
       <c r="C11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Không có</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n"/>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
-      <c r="H11" s="9" t="n"/>
+      <c r="H11" s="8" t="n">
+        <v>400000000</v>
+      </c>
       <c r="I11" s="4">
         <f>IF(H11="","",C11*H11)</f>
         <v/>
       </c>
-      <c r="J11" s="4" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>250 – 600 triệu</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Không có hệ nước siêu sạch trong hai tệp.</t>
+          <t>Hệ nước siêu sạch loại I (18,2 MΩ·cm) kèm tiền xử lý RO, 10–15 L/giờ, hãng châu Âu/Mỹ. Hãng Trung Quốc: khoảng 80–150 triệu.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1171,7 +1179,7 @@
         <f>IF(H12="","",C12*H12)</f>
         <v/>
       </c>
-      <c r="J12" s="4" t="n"/>
+      <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Eyela N-1300V-WB, bộ gồm bơm chân không và bộ làm lạnh; khắc phục thiếu sót phạm vi cung cấp đã nêu.</t>
@@ -1200,23 +1208,33 @@
       <c r="C13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Không có</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n"/>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
-      <c r="H13" s="9" t="n"/>
+      <c r="H13" s="8" t="n">
+        <v>250000000</v>
+      </c>
       <c r="I13" s="4">
         <f>IF(H13="","",C13*H13)</f>
         <v/>
       </c>
-      <c r="J13" s="4" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>150 – 350 triệu</t>
+        </is>
+      </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>"Lò thủy nhiệt" trong tệp là bể ổn nhiệt Memmert WNB, không phải bình phản ứng áp suất.</t>
+          <t>Thiết bị phản ứng áp suất 500 mL có khuấy, điều khiển nhiệt độ, đồng hồ áp suất, lót PPL (hãng Trung Quốc). Nếu chỉ là bình thủy nhiệt lót PPL: 10–20 triệu/bình. Loại Parr (Mỹ, Net-zero STT 19): khoảng 0,8–1 tỷ.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1242,23 +1260,33 @@
       <c r="C14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Không có</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n"/>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
-      <c r="H14" s="9" t="n"/>
+      <c r="H14" s="8" t="n">
+        <v>450000000</v>
+      </c>
       <c r="I14" s="4">
         <f>IF(H14="","",C14*H14)</f>
         <v/>
       </c>
-      <c r="J14" s="4" t="n"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>50 – 600 triệu</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Chỉ có hệ chiết công nghiệp 1.000 L (xưởng), không tương đương.</t>
+          <t>Giả định hệ chiết Soxhlet tự động 6 vị trí (châu Âu). Bộ Soxhlet thủy tinh + bếp 6 vị trí: 50–80 triệu; giá chiết pha rắn (SPE) 12 vị trí: 30–50 triệu. Cần xác định loại trước khi chốt.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1307,7 +1335,7 @@
         <f>IF(H15="","",C15*H15)</f>
         <v/>
       </c>
-      <c r="J15" s="4" t="n"/>
+      <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Máy UV-Vis Shimadzu UV-1800 (hai chùm tia), tương đương V-730.</t>
@@ -1336,23 +1364,33 @@
       <c r="C16" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Không có</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n"/>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
-      <c r="H16" s="9" t="n"/>
+      <c r="H16" s="8" t="n">
+        <v>2200000000</v>
+      </c>
       <c r="I16" s="4">
         <f>IF(H16="","",C16*H16)</f>
         <v/>
       </c>
-      <c r="J16" s="4" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>1.800 – 2.800 triệu</t>
+        </is>
+      </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Chỉ có GC-MS (5 tỷ), không có GC-FID/TCD.</t>
+          <t>GC-2030 với FID + TCD, bộ tiêm mẫu tự động, cột, phần mềm, máy tính, bình khí và van điều áp. Tham chiếu: GC-MS QP2020 NX trong tệp G9 là 5 tỷ.</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1405,7 +1443,7 @@
         <f>IF(H17="","",C17*H17)</f>
         <v/>
       </c>
-      <c r="J17" s="4" t="n"/>
+      <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Máy đo kích thước hạt, thế zeta (Zetasizer, NIBS). Đây là hạng mục đắt nhất đã có giá.</t>
@@ -1430,9 +1468,9 @@
       <c r="C18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Một phần</t>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Tương đồng</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1442,25 +1480,25 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Append1 / 47</t>
+          <t>Append1 / 188</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Máy sấy đông khô — BIOBASE BK -FD100S/Trung Quốc</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="n"/>
+          <t>Hệ thống đông khô — FDU-2110/Eyela/Nhật Bản Nhiệt độ bẫy lạnh: -80ºC, làm khô các mẫu với hàm lượng nước thấp Dung tích chứa đá (03L/một mẻ) Công suất làm lạnh: 500W x 02 • HFC (R4</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>900000000</v>
+      </c>
       <c r="I18" s="4">
         <f>IF(H18="","",C18*H18)</f>
         <v/>
       </c>
-      <c r="J18" s="4" t="n">
-        <v>430000000</v>
-      </c>
+      <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Máy đông khô Biobase BK-FD100S (loại pilot, lớn hơn FDL-2000 3 L/mẻ). Eyela FDU-2110 là 900 triệu. Chưa cộng vào tổng.</t>
+          <t>Eyela FDU-2110: bẫy lạnh -80 °C, 3 L/mẻ, bẫy đường kính 200 mm, trùng các thông số chính của FDL-2000. Giá cao; xem xét giảm còn 01 máy.</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1486,37 +1524,33 @@
       <c r="C19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Một phần</t>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Tệp 4_Thuốc</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>4 Thuốc / 47</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Máy đồng hoá siêu âm — Máy đồng hoá siêu âm</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="n"/>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="8" t="n">
+        <v>520000000</v>
+      </c>
       <c r="I19" s="4">
         <f>IF(H19="","",C19*H19)</f>
         <v/>
       </c>
-      <c r="J19" s="4" t="n">
-        <v>320000000</v>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>450 – 650 triệu</t>
+        </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Sonics VC505 (500 W), nhỏ hơn VCX 1500 (1.500 W). Chưa cộng vào tổng.</t>
+          <t>Quy đổi từ giá niêm yết VCX-1500-220 (kèm đầu dò, booster) 12.550 USD tại Mỹ, 14.100 EUR chưa VAT tại châu Âu; đối chiếu VC505 (500 W) = 320 triệu trong tệp 4_Thuốc.</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1569,7 +1603,7 @@
         <f>IF(H20="","",C20*H20)</f>
         <v/>
       </c>
-      <c r="J20" s="4" t="n"/>
+      <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Cùng model IKA T25 digital (giá ở sheet Append1).</t>
@@ -1621,7 +1655,7 @@
         <f>IF(H21="","",C21*H21)</f>
         <v/>
       </c>
-      <c r="J21" s="4" t="n"/>
+      <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Ly tâm lạnh đa năng 18.000 vòng/phút, 23.542 ×g, rotor 4 × 200 mL (Hermle Z327K).</t>
@@ -1646,37 +1680,33 @@
       <c r="C22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Một phần</t>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Tệp G9 (2025)</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>6 VLYS / 314</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Máy phân tích nhiệt TGA, DSC 1600oC (TGA/DSC 3+ - Thermogravimetric Analyzer with high temperature furnace (HT) — Hãng sx: Mettler- Toledo AG, Model: Analytical CH-8603 Schwerzenbach, Switzerland</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="n"/>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="8" t="n">
+        <v>3200000000</v>
+      </c>
       <c r="I22" s="4">
         <f>IF(H22="","",C22*H22)</f>
         <v/>
       </c>
-      <c r="J22" s="4" t="n">
-        <v>3696070000</v>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>2.800 – 4.500 triệu</t>
+        </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Chỉ có TGA/DSC 3+ Mettler (1600 °C), không có FTIR ghép nối; FTIR Bruker Vertex 70v ở Append1 là 1,2 tỷ. Chưa cộng vào tổng.</t>
+          <t>TGA tầm trung (~1,2–1,5 tỷ) + FTIR có ATR (~0,8–1 tỷ) + bộ ghép nối và phần mềm (~0,6–0,8 tỷ). Tham chiếu: TGA/DSC 3+ Mettler (1600 °C) = 3,70 tỷ; FTIR Bruker Vertex 70v = 1,2 tỷ (tệp G9).</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -1702,23 +1732,33 @@
       <c r="C23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Không có</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n"/>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
-      <c r="H23" s="9" t="n"/>
+      <c r="H23" s="8" t="n">
+        <v>1500000000</v>
+      </c>
       <c r="I23" s="4">
         <f>IF(H23="","",C23*H23)</f>
         <v/>
       </c>
-      <c r="J23" s="4" t="n"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>1.300 – 1.800 triệu</t>
+        </is>
+      </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Không có AAS.</t>
+          <t>AAS ngọn lửa hiệu chỉnh Zeeman, kèm máy nén khí, bình acetylen, đèn, chụp hút, máy tính.</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -1740,23 +1780,33 @@
       <c r="C24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Không có</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n"/>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
-      <c r="H24" s="9" t="n"/>
+      <c r="H24" s="8" t="n">
+        <v>800000000</v>
+      </c>
       <c r="I24" s="4">
         <f>IF(H24="","",C24*H24)</f>
         <v/>
       </c>
-      <c r="J24" s="4" t="n"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>300 – 1.300 triệu</t>
+        </is>
+      </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Không có máy kéo đa năng.</t>
+          <t>Máy thử kéo vạn năng điện cơ 5–10 kN: hãng Nhật/châu Âu khoảng 1,0–1,3 tỷ; hãng Trung Quốc 250–400 triệu. Cần xác định tải trọng.</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -1782,23 +1832,33 @@
       <c r="C25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Không có</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n"/>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
-      <c r="H25" s="9" t="n"/>
+      <c r="H25" s="8" t="n">
+        <v>300000000</v>
+      </c>
       <c r="I25" s="4">
         <f>IF(H25="","",C25*H25)</f>
         <v/>
       </c>
-      <c r="J25" s="4" t="n"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>200 – 450 triệu</t>
+        </is>
+      </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Không có máy đo độ dẫn 4 đầu.</t>
+          <t>Giả định máy đo điện trở mặt 4 mũi dò cho màng mỏng (có nguồn dòng, phần mềm). Nếu là máy đo độ dẫn dung dịch đa kênh: 50–100 triệu.</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -1847,7 +1907,7 @@
         <f>IF(H26="","",C26*H26)</f>
         <v/>
       </c>
-      <c r="J26" s="4" t="n"/>
+      <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Lò nung ống 2 vùng có bơm chân không (GSS70600, Hàn Quốc); giá có thể cao hơn lò KJ (Trung Quốc).</t>
@@ -1876,23 +1936,33 @@
       <c r="C27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Không có</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n"/>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
-      <c r="H27" s="9" t="n"/>
+      <c r="H27" s="8" t="n">
+        <v>3000000000</v>
+      </c>
       <c r="I27" s="4">
         <f>IF(H27="","",C27*H27)</f>
         <v/>
       </c>
-      <c r="J27" s="4" t="n"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>2.500 – 3.500 triệu</t>
+        </is>
+      </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Chỉ có máy đo độ tan rã thuốc (60 triệu), khác thiết bị đo độ hòa tan.</t>
+          <t>708-DS 8 vị trí + 850-DS lấy mẫu tự động + UV-Vis đo trực tuyến và phần mềm. Không kèm UV-Vis: khoảng 2,0 tỷ.</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -1914,37 +1984,33 @@
       <c r="C28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>Một phần</t>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Tệp G9 (2025)</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Append1 / 901</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>CS350M Potentiostat/Galvan ostat with EIS — Potential Control: ±10 V (customizable to ±12 V) Current Control: ±2 A, 10 automatic ranges (2 nA - 2 A) Compliance Voltage: ±21 V Accuracy: 0.1 % of full range</t>
-        </is>
-      </c>
-      <c r="H28" s="7" t="n"/>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="8" t="n">
+        <v>500000000</v>
+      </c>
       <c r="I28" s="4">
         <f>IF(H28="","",C28*H28)</f>
         <v/>
       </c>
-      <c r="J28" s="4" t="n">
-        <v>80000000</v>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>400 – 650 triệu</t>
+        </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Corrtest CS350M, 1 kênh có EIS, 80 triệu; đề cương là hệ 8 kênh. Chưa cộng vào tổng.</t>
+          <t>Corrtest CS310X Option C (8 kênh, 1 kênh EIS; model có thật theo catalogue hãng). Đối chiếu: CS350M 1 kênh EIS = 80 triệu (tệp G9).</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -1970,23 +2036,33 @@
       <c r="C29" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Không có</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n"/>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Ước lượng thị trường VN</t>
+        </is>
+      </c>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
-      <c r="H29" s="9" t="n"/>
+      <c r="H29" s="8" t="n">
+        <v>1500000000</v>
+      </c>
       <c r="I29" s="4">
         <f>IF(H29="","",C29*H29)</f>
         <v/>
       </c>
-      <c r="J29" s="4" t="n"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>1.000 – 3.000 triệu</t>
+        </is>
+      </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Không có máy huỳnh quang/PL (chỉ có máy đọc vi đĩa, kính hiển vi huỳnh quang).</t>
+          <t>Máy huỳnh quang để bàn đèn Xe, có giá đo mẫu rắn (tầm trung). Dòng cao cấp (Horiba FluoroMax Plus): 2,5–3,0 tỷ.</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2002,9 +2078,9 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr"/>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>TỔNG các hạng mục đã có giá tạm</t>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>TỔNG (giá danh mục + giá liên quan + ước lượng)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr"/>
@@ -2013,27 +2089,20 @@
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" s="11">
+      <c r="I30" s="10">
         <f>SUM(I2:I29)</f>
         <v/>
       </c>
-      <c r="J30" s="4">
-        <f>SUMPRODUCT(C2:C29,J2:J29)</f>
-        <v/>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Cột J: tổng nếu lấy cả giá "Một phần" (nhân số lượng)</t>
-        </is>
-      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="n"/>
       <c r="M30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr"/>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Số hạng mục chưa có giá tạm</t>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Trong đó: phần ước lượng</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr"/>
@@ -2042,18 +2111,18 @@
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="11">
-        <f>COUNTBLANK(H2:H29)</f>
-        <v/>
-      </c>
-      <c r="J31" s="4" t="inlineStr"/>
+      <c r="I31" s="10">
+        <f>SUMIF(D2:D29,"Ước lượng",I2:I29)</f>
+        <v/>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="n"/>
       <c r="M31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr"/>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Tổng kinh phí tối đa</t>
         </is>
@@ -2064,19 +2133,19 @@
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr"/>
-      <c r="I32" s="11" t="n">
+      <c r="I32" s="10" t="n">
         <v>15000000000</v>
       </c>
-      <c r="J32" s="4" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="n"/>
       <c r="M32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr"/>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>Còn lại cho các hạng mục chưa có giá và hạng mục bổ sung</t>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Chênh lệch (âm = vượt)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr"/>
@@ -2085,11 +2154,11 @@
       <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" s="11">
+      <c r="I33" s="10">
         <f>I32-I30</f>
         <v/>
       </c>
-      <c r="J33" s="4" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr"/>
       <c r="L33" s="2" t="n"/>
       <c r="M33" s="2" t="n"/>
@@ -2100,6 +2169,1301 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="58" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Thiết bị</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>SL đề cương</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Đơn giá tạm (đồng)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Thành tiền theo đề cương</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>SL đề xuất</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Đơn giá đề xuất (đồng)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Thành tiền theo đề xuất</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Chênh lệch</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Lý do điều chỉnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Tủ hút Phượng Hải - Việt Nam</t>
+        </is>
+      </c>
+      <c r="C2" s="2">
+        <f>'Đối sánh giá'!C2</f>
+        <v/>
+      </c>
+      <c r="D2" s="4">
+        <f>'Đối sánh giá'!H2</f>
+        <v/>
+      </c>
+      <c r="E2" s="4">
+        <f>C2*D2</f>
+        <v/>
+      </c>
+      <c r="F2" s="2">
+        <f>C2</f>
+        <v/>
+      </c>
+      <c r="G2" s="4">
+        <f>D2</f>
+        <v/>
+      </c>
+      <c r="H2" s="4">
+        <f>F2*G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="4">
+        <f>H2-E2</f>
+        <v/>
+      </c>
+      <c r="J2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Cân 4 số BCE224i-1S Sartorius - Trung Quốc</t>
+        </is>
+      </c>
+      <c r="C3" s="2">
+        <f>'Đối sánh giá'!C3</f>
+        <v/>
+      </c>
+      <c r="D3" s="4">
+        <f>'Đối sánh giá'!H3</f>
+        <v/>
+      </c>
+      <c r="E3" s="4">
+        <f>C3*D3</f>
+        <v/>
+      </c>
+      <c r="F3" s="2">
+        <f>C3</f>
+        <v/>
+      </c>
+      <c r="G3" s="4">
+        <f>D3</f>
+        <v/>
+      </c>
+      <c r="H3" s="4">
+        <f>F3*G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="4">
+        <f>H3-E3</f>
+        <v/>
+      </c>
+      <c r="J3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Cân 2 số SPX6201 Ohaus - Trung Quốc</t>
+        </is>
+      </c>
+      <c r="C4" s="2">
+        <f>'Đối sánh giá'!C4</f>
+        <v/>
+      </c>
+      <c r="D4" s="4">
+        <f>'Đối sánh giá'!H4</f>
+        <v/>
+      </c>
+      <c r="E4" s="4">
+        <f>C4*D4</f>
+        <v/>
+      </c>
+      <c r="F4" s="2">
+        <f>C4</f>
+        <v/>
+      </c>
+      <c r="G4" s="4">
+        <f>D4</f>
+        <v/>
+      </c>
+      <c r="H4" s="4">
+        <f>F4*G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="4">
+        <f>H4-E4</f>
+        <v/>
+      </c>
+      <c r="J4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Máy khuấy từ gia nhiệt AREC 7 Velp - Ý</t>
+        </is>
+      </c>
+      <c r="C5" s="2">
+        <f>'Đối sánh giá'!C5</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>'Đối sánh giá'!H5</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>C5*D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="2">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>D5</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>F5*G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="4">
+        <f>H5-E5</f>
+        <v/>
+      </c>
+      <c r="J5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Bể rửa siêu âm thể tích 6 lít Model: WUC-D06H Hãng sản xuất: Daihan - Hàn Quốc</t>
+        </is>
+      </c>
+      <c r="C6" s="2">
+        <f>'Đối sánh giá'!C6</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>'Đối sánh giá'!H6</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>C6*D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="2">
+        <f>C6</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
+        <f>D6</f>
+        <v/>
+      </c>
+      <c r="H6" s="4">
+        <f>F6*G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="4">
+        <f>H6-E6</f>
+        <v/>
+      </c>
+      <c r="J6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Tủ sấy UN55 Memmert - Đức</t>
+        </is>
+      </c>
+      <c r="C7" s="2">
+        <f>'Đối sánh giá'!C7</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>'Đối sánh giá'!H7</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>C7*D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="2">
+        <f>C7</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>D7</f>
+        <v/>
+      </c>
+      <c r="H7" s="4">
+        <f>F7*G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="4">
+        <f>H7-E7</f>
+        <v/>
+      </c>
+      <c r="J7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tủ lạnh Hòa Phát - Việt Nam</t>
+        </is>
+      </c>
+      <c r="C8" s="2">
+        <f>'Đối sánh giá'!C8</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>'Đối sánh giá'!H8</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="2">
+        <f>C8</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>D8</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>F8*G8</f>
+        <v/>
+      </c>
+      <c r="I8" s="4">
+        <f>H8-E8</f>
+        <v/>
+      </c>
+      <c r="J8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Tủ đông Hòa Phát - Việt Nam</t>
+        </is>
+      </c>
+      <c r="C9" s="2">
+        <f>'Đối sánh giá'!C9</f>
+        <v/>
+      </c>
+      <c r="D9" s="4">
+        <f>'Đối sánh giá'!H9</f>
+        <v/>
+      </c>
+      <c r="E9" s="4">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="2">
+        <f>C9</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>D9</f>
+        <v/>
+      </c>
+      <c r="H9" s="4">
+        <f>F9*G9</f>
+        <v/>
+      </c>
+      <c r="I9" s="4">
+        <f>H9-E9</f>
+        <v/>
+      </c>
+      <c r="J9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Máy chưng cất nước 2 lần Model: WSC/4D Hãng sản xuất: HAMILTON - Anh</t>
+        </is>
+      </c>
+      <c r="C10" s="2">
+        <f>'Đối sánh giá'!C10</f>
+        <v/>
+      </c>
+      <c r="D10" s="4">
+        <f>'Đối sánh giá'!H10</f>
+        <v/>
+      </c>
+      <c r="E10" s="4">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="2">
+        <f>C10</f>
+        <v/>
+      </c>
+      <c r="G10" s="4">
+        <f>D10</f>
+        <v/>
+      </c>
+      <c r="H10" s="4">
+        <f>F10*G10</f>
+        <v/>
+      </c>
+      <c r="I10" s="4">
+        <f>H10-E10</f>
+        <v/>
+      </c>
+      <c r="J10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Hệ nước siêu sạch</t>
+        </is>
+      </c>
+      <c r="C11" s="2">
+        <f>'Đối sánh giá'!C11</f>
+        <v/>
+      </c>
+      <c r="D11" s="4">
+        <f>'Đối sánh giá'!H11</f>
+        <v/>
+      </c>
+      <c r="E11" s="4">
+        <f>C11*D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="2">
+        <f>C11</f>
+        <v/>
+      </c>
+      <c r="G11" s="4">
+        <f>D11</f>
+        <v/>
+      </c>
+      <c r="H11" s="4">
+        <f>F11*G11</f>
+        <v/>
+      </c>
+      <c r="I11" s="4">
+        <f>H11-E11</f>
+        <v/>
+      </c>
+      <c r="J11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Máy cô quay chân không và phụ kiện Model: N-1300E-W Hãng sản xuất: Tokyo Rikakikai (Eyela) - Nhật Bản</t>
+        </is>
+      </c>
+      <c r="C12" s="2">
+        <f>'Đối sánh giá'!C12</f>
+        <v/>
+      </c>
+      <c r="D12" s="4">
+        <f>'Đối sánh giá'!H12</f>
+        <v/>
+      </c>
+      <c r="E12" s="4">
+        <f>C12*D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="2">
+        <f>C12</f>
+        <v/>
+      </c>
+      <c r="G12" s="4">
+        <f>D12</f>
+        <v/>
+      </c>
+      <c r="H12" s="4">
+        <f>F12*G12</f>
+        <v/>
+      </c>
+      <c r="I12" s="4">
+        <f>H12-E12</f>
+        <v/>
+      </c>
+      <c r="J12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Hệ phản ứng kiểm soát nhiệt, áp suất Model: TOP-HP500 Hãng sản xuất: Toption - Trung Quốc</t>
+        </is>
+      </c>
+      <c r="C13" s="2">
+        <f>'Đối sánh giá'!C13</f>
+        <v/>
+      </c>
+      <c r="D13" s="4">
+        <f>'Đối sánh giá'!H13</f>
+        <v/>
+      </c>
+      <c r="E13" s="4">
+        <f>C13*D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="2">
+        <f>C13</f>
+        <v/>
+      </c>
+      <c r="G13" s="4">
+        <f>D13</f>
+        <v/>
+      </c>
+      <c r="H13" s="4">
+        <f>F13*G13</f>
+        <v/>
+      </c>
+      <c r="I13" s="4">
+        <f>H13-E13</f>
+        <v/>
+      </c>
+      <c r="J13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Hệ chiết tách</t>
+        </is>
+      </c>
+      <c r="C14" s="2">
+        <f>'Đối sánh giá'!C14</f>
+        <v/>
+      </c>
+      <c r="D14" s="4">
+        <f>'Đối sánh giá'!H14</f>
+        <v/>
+      </c>
+      <c r="E14" s="4">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="2">
+        <f>C14</f>
+        <v/>
+      </c>
+      <c r="G14" s="4">
+        <f>D14</f>
+        <v/>
+      </c>
+      <c r="H14" s="4">
+        <f>F14*G14</f>
+        <v/>
+      </c>
+      <c r="I14" s="4">
+        <f>H14-E14</f>
+        <v/>
+      </c>
+      <c r="J14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Máy quang phổ UV-Vis V730 Jasco - Nhật</t>
+        </is>
+      </c>
+      <c r="C15" s="2">
+        <f>'Đối sánh giá'!C15</f>
+        <v/>
+      </c>
+      <c r="D15" s="4">
+        <f>'Đối sánh giá'!H15</f>
+        <v/>
+      </c>
+      <c r="E15" s="4">
+        <f>C15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="8">
+        <f>D15</f>
+        <v/>
+      </c>
+      <c r="H15" s="4">
+        <f>F15*G15</f>
+        <v/>
+      </c>
+      <c r="I15" s="4">
+        <f>H15-E15</f>
+        <v/>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Giữ 01 UV-Vis; Khoa nhiều khả năng đã có UV-Vis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Máy sắc ký khí (đầu dò FID, TCD) Model: GC-2030 Hãng sản xuất: Shimadzu - Nhật</t>
+        </is>
+      </c>
+      <c r="C16" s="2">
+        <f>'Đối sánh giá'!C16</f>
+        <v/>
+      </c>
+      <c r="D16" s="4">
+        <f>'Đối sánh giá'!H16</f>
+        <v/>
+      </c>
+      <c r="E16" s="4">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="2">
+        <f>C16</f>
+        <v/>
+      </c>
+      <c r="G16" s="4">
+        <f>D16</f>
+        <v/>
+      </c>
+      <c r="H16" s="4">
+        <f>F16*G16</f>
+        <v/>
+      </c>
+      <c r="I16" s="4">
+        <f>H16-E16</f>
+        <v/>
+      </c>
+      <c r="J16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Thiết Bị Đo Kích Thước Hạt và Thế Zeta (Zetasizer Advance Range) Malvern Panalytical Model Zetasizer Pro</t>
+        </is>
+      </c>
+      <c r="C17" s="2">
+        <f>'Đối sánh giá'!C17</f>
+        <v/>
+      </c>
+      <c r="D17" s="4">
+        <f>'Đối sánh giá'!H17</f>
+        <v/>
+      </c>
+      <c r="E17" s="4">
+        <f>C17*D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="8">
+        <f>D17</f>
+        <v/>
+      </c>
+      <c r="H17" s="4">
+        <f>F17*G17</f>
+        <v/>
+      </c>
+      <c r="I17" s="4">
+        <f>H17-E17</f>
+        <v/>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>Máy đo kích thước hạt, thế zeta chiếm khoảng 4,4 tỷ. Bỏ nếu kiểm kê cho thấy Trường hoặc ĐHQG-HCM đã có thiết bị DLS dùng chung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Tủ sấy đông khô Model: FDL-2000 Hãng sản xuất: Eyela - Nhật</t>
+        </is>
+      </c>
+      <c r="C18" s="2">
+        <f>'Đối sánh giá'!C18</f>
+        <v/>
+      </c>
+      <c r="D18" s="4">
+        <f>'Đối sánh giá'!H18</f>
+        <v/>
+      </c>
+      <c r="E18" s="4">
+        <f>C18*D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="8">
+        <f>D18</f>
+        <v/>
+      </c>
+      <c r="H18" s="4">
+        <f>F18*G18</f>
+        <v/>
+      </c>
+      <c r="I18" s="4">
+        <f>H18-E18</f>
+        <v/>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>Hai máy đông khô cần lý giải bằng số mẫu; giữ 01 máy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Máy đồng nhất siêu âm dạng thanh Model: VCX 1500 Hãng sản xuất: Sonics - Mỹ</t>
+        </is>
+      </c>
+      <c r="C19" s="2">
+        <f>'Đối sánh giá'!C19</f>
+        <v/>
+      </c>
+      <c r="D19" s="4">
+        <f>'Đối sánh giá'!H19</f>
+        <v/>
+      </c>
+      <c r="E19" s="4">
+        <f>C19*D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="2">
+        <f>C19</f>
+        <v/>
+      </c>
+      <c r="G19" s="4">
+        <f>D19</f>
+        <v/>
+      </c>
+      <c r="H19" s="4">
+        <f>F19*G19</f>
+        <v/>
+      </c>
+      <c r="I19" s="4">
+        <f>H19-E19</f>
+        <v/>
+      </c>
+      <c r="J19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Máy đồng hóa tốc độ cao T25 digital ultra-turrax IKA - Đức</t>
+        </is>
+      </c>
+      <c r="C20" s="2">
+        <f>'Đối sánh giá'!C20</f>
+        <v/>
+      </c>
+      <c r="D20" s="4">
+        <f>'Đối sánh giá'!H20</f>
+        <v/>
+      </c>
+      <c r="E20" s="4">
+        <f>C20*D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="2">
+        <f>C20</f>
+        <v/>
+      </c>
+      <c r="G20" s="4">
+        <f>D20</f>
+        <v/>
+      </c>
+      <c r="H20" s="4">
+        <f>F20*G20</f>
+        <v/>
+      </c>
+      <c r="I20" s="4">
+        <f>H20-E20</f>
+        <v/>
+      </c>
+      <c r="J20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Máy ly tâm tốc độ cao (có làm lạnh) Model: Z032-HK-E Hãng sản xuất: HERMLE - Benchmark</t>
+        </is>
+      </c>
+      <c r="C21" s="2">
+        <f>'Đối sánh giá'!C21</f>
+        <v/>
+      </c>
+      <c r="D21" s="4">
+        <f>'Đối sánh giá'!H21</f>
+        <v/>
+      </c>
+      <c r="E21" s="4">
+        <f>C21*D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="2">
+        <f>C21</f>
+        <v/>
+      </c>
+      <c r="G21" s="4">
+        <f>D21</f>
+        <v/>
+      </c>
+      <c r="H21" s="4">
+        <f>F21*G21</f>
+        <v/>
+      </c>
+      <c r="I21" s="4">
+        <f>H21-E21</f>
+        <v/>
+      </c>
+      <c r="J21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Máy TGA-FTIR</t>
+        </is>
+      </c>
+      <c r="C22" s="2">
+        <f>'Đối sánh giá'!C22</f>
+        <v/>
+      </c>
+      <c r="D22" s="4">
+        <f>'Đối sánh giá'!H22</f>
+        <v/>
+      </c>
+      <c r="E22" s="4">
+        <f>C22*D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="H22" s="4">
+        <f>F22*G22</f>
+        <v/>
+      </c>
+      <c r="I22" s="4">
+        <f>H22-E22</f>
+        <v/>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>Hạ cấu hình: chỉ mua TGA (hoặc TGA/DSC tầm trung), dùng FTIR sẵn có của Khoa. Đơn giá đề xuất là ước lượng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Máy quang phổ hấp thụ nguyên tử ZA4300 Hitachi - Nhật</t>
+        </is>
+      </c>
+      <c r="C23" s="2">
+        <f>'Đối sánh giá'!C23</f>
+        <v/>
+      </c>
+      <c r="D23" s="4">
+        <f>'Đối sánh giá'!H23</f>
+        <v/>
+      </c>
+      <c r="E23" s="4">
+        <f>C23*D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="2">
+        <f>C23</f>
+        <v/>
+      </c>
+      <c r="G23" s="4">
+        <f>D23</f>
+        <v/>
+      </c>
+      <c r="H23" s="4">
+        <f>F23*G23</f>
+        <v/>
+      </c>
+      <c r="I23" s="4">
+        <f>H23-E23</f>
+        <v/>
+      </c>
+      <c r="J23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Máy đo kéo đa năng</t>
+        </is>
+      </c>
+      <c r="C24" s="2">
+        <f>'Đối sánh giá'!C24</f>
+        <v/>
+      </c>
+      <c r="D24" s="4">
+        <f>'Đối sánh giá'!H24</f>
+        <v/>
+      </c>
+      <c r="E24" s="4">
+        <f>C24*D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="2">
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="G24" s="4">
+        <f>D24</f>
+        <v/>
+      </c>
+      <c r="H24" s="4">
+        <f>F24*G24</f>
+        <v/>
+      </c>
+      <c r="I24" s="4">
+        <f>H24-E24</f>
+        <v/>
+      </c>
+      <c r="J24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Máy đo độ dẫn đa năng 4 đầu</t>
+        </is>
+      </c>
+      <c r="C25" s="2">
+        <f>'Đối sánh giá'!C25</f>
+        <v/>
+      </c>
+      <c r="D25" s="4">
+        <f>'Đối sánh giá'!H25</f>
+        <v/>
+      </c>
+      <c r="E25" s="4">
+        <f>C25*D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="2">
+        <f>C25</f>
+        <v/>
+      </c>
+      <c r="G25" s="4">
+        <f>D25</f>
+        <v/>
+      </c>
+      <c r="H25" s="4">
+        <f>F25*G25</f>
+        <v/>
+      </c>
+      <c r="I25" s="4">
+        <f>H25-E25</f>
+        <v/>
+      </c>
+      <c r="J25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Lò nung ống Model: KJ-TCVD1200-S80LK2W Hãng sản xuất: KJ Technology - TQ</t>
+        </is>
+      </c>
+      <c r="C26" s="2">
+        <f>'Đối sánh giá'!C26</f>
+        <v/>
+      </c>
+      <c r="D26" s="4">
+        <f>'Đối sánh giá'!H26</f>
+        <v/>
+      </c>
+      <c r="E26" s="4">
+        <f>C26*D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="8">
+        <f>D26</f>
+        <v/>
+      </c>
+      <c r="H26" s="4">
+        <f>F26*G26</f>
+        <v/>
+      </c>
+      <c r="I26" s="4">
+        <f>H26-E26</f>
+        <v/>
+      </c>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>Giữ 01 lò ống; bổ sung 01 lò nung buồng (sheet Đề xuất bổ sung).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống máy đo độ hòa tan, 8 vị trí + hệ thống lấy mẫu tự động 708-DS Dissolution Apparatus, 8-position Agilent - Mỹ</t>
+        </is>
+      </c>
+      <c r="C27" s="2">
+        <f>'Đối sánh giá'!C27</f>
+        <v/>
+      </c>
+      <c r="D27" s="4">
+        <f>'Đối sánh giá'!H27</f>
+        <v/>
+      </c>
+      <c r="E27" s="4">
+        <f>C27*D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="8">
+        <f>D27</f>
+        <v/>
+      </c>
+      <c r="H27" s="4">
+        <f>F27*G27</f>
+        <v/>
+      </c>
+      <c r="I27" s="4">
+        <f>H27-E27</f>
+        <v/>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>Thiết bị kiểm nghiệm dược (QC), ít gắn với nghiên cứu hóa học chung; giá cao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Bộ điều chỉnh điện áp đa kênh gồm 8 kênh, EIS*1 Ký mã hiệu: CS310X (Option C, 8-channel, EIS*1) Hãng sản xuất: Corrtest Xuất xứ: Trung Quốc</t>
+        </is>
+      </c>
+      <c r="C28" s="2">
+        <f>'Đối sánh giá'!C28</f>
+        <v/>
+      </c>
+      <c r="D28" s="4">
+        <f>'Đối sánh giá'!H28</f>
+        <v/>
+      </c>
+      <c r="E28" s="4">
+        <f>C28*D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="2">
+        <f>C28</f>
+        <v/>
+      </c>
+      <c r="G28" s="4">
+        <f>D28</f>
+        <v/>
+      </c>
+      <c r="H28" s="4">
+        <f>F28*G28</f>
+        <v/>
+      </c>
+      <c r="I28" s="4">
+        <f>H28-E28</f>
+        <v/>
+      </c>
+      <c r="J28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Máy đo phổ quang phát quang PL</t>
+        </is>
+      </c>
+      <c r="C29" s="2">
+        <f>'Đối sánh giá'!C29</f>
+        <v/>
+      </c>
+      <c r="D29" s="4">
+        <f>'Đối sánh giá'!H29</f>
+        <v/>
+      </c>
+      <c r="E29" s="4">
+        <f>C29*D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="2">
+        <f>C29</f>
+        <v/>
+      </c>
+      <c r="G29" s="4">
+        <f>D29</f>
+        <v/>
+      </c>
+      <c r="H29" s="4">
+        <f>F29*G29</f>
+        <v/>
+      </c>
+      <c r="I29" s="4">
+        <f>H29-E29</f>
+        <v/>
+      </c>
+      <c r="J29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Cộng danh mục</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="4" t="inlineStr"/>
+      <c r="E30" s="4">
+        <f>SUM(E2:E29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr"/>
+      <c r="H30" s="4">
+        <f>SUM(H2:H29)</f>
+        <v/>
+      </c>
+      <c r="I30" s="4">
+        <f>SUM(I2:I29)</f>
+        <v/>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr"/>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Cộng nhóm "Nên bổ sung" (sheet Đề xuất bổ sung)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4">
+        <f>'Đề xuất bổ sung'!H10</f>
+        <v/>
+      </c>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>TỔNG</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="4" t="inlineStr"/>
+      <c r="E32" s="4">
+        <f>E30</f>
+        <v/>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="4">
+        <f>H30+H31</f>
+        <v/>
+      </c>
+      <c r="I32" s="4" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Tổng kinh phí tối đa</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="n">
+        <v>15000000000</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="n">
+        <v>15000000000</v>
+      </c>
+      <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr"/>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Chênh lệch (âm = vượt)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr"/>
+      <c r="E34" s="4">
+        <f>E33-E32</f>
+        <v/>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr"/>
+      <c r="H34" s="4">
+        <f>H33-H32</f>
+        <v/>
+      </c>
+      <c r="I34" s="4" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2527,13 +3891,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2541,98 +3905,110 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Mục</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Nội dung</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Nguồn giá</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>(1) Tệp "4_Thuốc": đơn giá sau thuế, bản đã cắt giảm (ưu tiên sử dụng). (2) Tệp "Danh mục thiết bị G9 ... 09.08 sau khi giảm bớt": các sheet theo phòng thí nghiệm (cập nhật 05/08/2025) và sheet tổng hợp Append1 (giá số tròn, bản đề xuất ban đầu). Thứ tự ưu tiên: 4_Thuốc &gt; sheet theo phòng thí nghiệm &gt; Append1.</t>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>(1) Tệp "4_Thuốc": đơn giá sau thuế, bản đã cắt giảm (ưu tiên). (2) Tệp "Danh mục thiết bị G9 ... 09.08 sau khi giảm bớt": sheet theo phòng thí nghiệm (cập nhật 05/08/2025) và sheet tổng hợp Append1 (số tròn, đề xuất ban đầu). Thứ tự ưu tiên: 4_Thuốc &gt; sheet theo phòng thí nghiệm &gt; Append1.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Trùng model</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Cùng model trong danh mục tham chiếu: dùng đơn giá.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Tương đồng</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Cùng loại, cấu hình gần tương đương: dùng làm giá tạm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Giá liên quan</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Thiết bị liên quan trong danh mục tham chiếu, theo phương án đã góp ý (ví dụ tủ âm -30 °C thay tủ đông gia dụng).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Ước lượng</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Không có trong danh mục tham chiếu. Đơn giá là ước lượng của người lập bảng theo mặt bằng giá thiết bị cùng loại trong tệp G9/4_Thuốc và giá niêm yết quốc tế (quy đổi khoảng 1,3–1,6 × giá USD × 26.000 đ/USD cho nhập khẩu, VAT, lắp đặt, đào tạo). Chỉ dùng để cân đối danh mục; không dùng làm căn cứ dự toán. Cần tối thiểu 03 báo giá.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Giới hạn tra cứu</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Các cổng muasamcong.mpi.gov.vn và dauthau.asia không truy cập được từ môi trường làm việc, nên chưa đối chiếu được giá trúng thầu. Giá niêm yết tìm được: Sonics VCX-1500-220 12.550 USD (John Morris Group, Mỹ); 14.100 EUR chưa VAT (Spectratech, Hy Lạp).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Thời điểm giá</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Giá thuộc năm 2025; cần cập nhật báo giá năm 2026 trước khi lập dự toán chính thức.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Trùng model</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Cùng model: dùng đơn giá.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Tương đồng</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Cùng loại, cấu hình gần tương đương: dùng làm giá tạm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Một phần</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Cùng nhóm nhưng khác cấu hình đáng kể: ghi ở cột "Giá tham khảo", không cộng vào tổng; cần quyết định.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Không có</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Không có trong hai tệp: để trống, cần tìm báo giá.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Giá tệp G9/4_Thuốc thuộc năm 2025; cần cập nhật báo giá 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Hệ máy tính đã bỏ</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Tệp 4_Thuốc có "Hệ thống máy vi tính hiệu năng cao chuyên dụng" 542.860.000 đồng; đây là mức kinh phí tham khảo tiết kiệm được khi bỏ hạng mục hệ máy tính.</t>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Tệp 4_Thuốc có "Hệ thống máy vi tính hiệu năng cao chuyên dụng" 542.860.000 đồng: mức tham khảo cho khoản đã tiết kiệm.</t>
         </is>
       </c>
     </row>

</xml_diff>